<commit_message>
paper run 2026-09-14 17:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-14.xlsx
+++ b/reports/2026-09-14.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,135 @@
       </c>
       <c r="K2" t="n">
         <v>7.99</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-14T13:41:17.080369+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.00155</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-14T13:56:16.984324+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F4" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>25.18</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.00118</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>11.08</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-14T14:41:48.890839+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F5" t="n">
+        <v>48.13</v>
+      </c>
+      <c r="G5" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00105</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>39.37</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +679,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +689,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -570,7 +699,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -580,7 +709,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="6">
@@ -590,7 +719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.99</v>
+        <v>28.44</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +729,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.99</v>
+        <v>58.44</v>
       </c>
     </row>
     <row r="8">
@@ -610,7 +739,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="9">
@@ -620,7 +749,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="10">
@@ -630,7 +759,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>991.8299999999999</v>
+        <v>1012.28</v>
       </c>
     </row>
     <row r="12">
@@ -681,16 +810,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>-1.65</v>
+        <v>11.37</v>
       </c>
       <c r="E15" t="n">
-        <v>7.99</v>
+        <v>28.44</v>
       </c>
     </row>
     <row r="16">
@@ -700,13 +829,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>64.34999999999999</v>
+        <v>114.97</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -726,51 +855,51 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>38.65</v>
+        <v>29.93</v>
       </c>
       <c r="E18" t="n">
-        <v>7.99</v>
+        <v>47.36</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>-40.3</v>
+        <v>0.31</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>64.34999999999999</v>
+        <v>43.21</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -779,69 +908,81 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="n">
+        <v>52.89</v>
+      </c>
+      <c r="E21" t="n">
+        <v>11.08</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>3</v>
-      </c>
-      <c r="C22" t="n">
-        <v>3</v>
-      </c>
-      <c r="D22" t="n">
-        <v>103</v>
-      </c>
-      <c r="E22" t="n">
-        <v>7.99</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D23" t="n">
-        <v>-40.3</v>
+        <v>120.31</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>46.33</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-10.93</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>24.05</v>
+        <v>-40.3</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -850,71 +991,78 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" t="n">
-        <v>38.65</v>
-      </c>
-      <c r="E26" t="n">
-        <v>7.99</v>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-53.42</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" t="n">
+        <v>110.32</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="E29" t="n">
+        <v>28.44</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BTC</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>7.99</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>По окнам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -936,169 +1084,303 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>7.99</v>
+        <v>47.36</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-30</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>11.08</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>7.99</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="n">
+        <v>28.44</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>7.99</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>7.99</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C43" t="n">
         <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>7.99</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>-18.92</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>39.37</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>39.37</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-10.93</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>3</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>58.44</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="n">
-        <v>7.99</v>
+      <c r="B55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" t="n">
+        <v>3</v>
+      </c>
+      <c r="D55" t="n">
+        <v>28.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-14 23:53
</commit_message>
<xml_diff>
--- a/reports/2026-09-14.xlsx
+++ b/reports/2026-09-14.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,49 @@
       </c>
       <c r="K5" t="n">
         <v>39.37</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-14T19:27:01.383943+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F6" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>25</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.819</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.00263</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>11.5</v>
       </c>
     </row>
   </sheetData>
@@ -657,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,7 +722,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -689,7 +732,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -709,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6">
@@ -719,7 +762,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28.44</v>
+        <v>39.94</v>
       </c>
     </row>
     <row r="7">
@@ -729,7 +772,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58.44</v>
+        <v>69.94</v>
       </c>
     </row>
     <row r="8">
@@ -749,7 +792,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.95</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="10">
@@ -759,7 +802,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1012.28</v>
+        <v>1023.78</v>
       </c>
     </row>
     <row r="12">
@@ -810,16 +853,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>11.37</v>
+        <v>-41.41</v>
       </c>
       <c r="E15" t="n">
-        <v>28.44</v>
+        <v>39.94</v>
       </c>
     </row>
     <row r="16">
@@ -829,13 +872,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>114.97</v>
+        <v>191.02</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -893,13 +936,13 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="n">
         <v>3</v>
       </c>
-      <c r="C20" t="n">
-        <v>2</v>
-      </c>
       <c r="D20" t="n">
-        <v>43.21</v>
+        <v>73.87</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -912,16 +955,16 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" t="n">
         <v>6</v>
       </c>
-      <c r="C21" t="n">
-        <v>4</v>
-      </c>
       <c r="D21" t="n">
-        <v>52.89</v>
+        <v>45.5</v>
       </c>
       <c r="E21" t="n">
-        <v>11.08</v>
+        <v>22.58</v>
       </c>
     </row>
     <row r="22">
@@ -938,16 +981,16 @@
         </is>
       </c>
       <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="n">
         <v>7</v>
       </c>
-      <c r="C23" t="n">
-        <v>5</v>
-      </c>
       <c r="D23" t="n">
-        <v>120.31</v>
+        <v>157.63</v>
       </c>
       <c r="E23" t="n">
-        <v>39.37</v>
+        <v>50.87</v>
       </c>
     </row>
     <row r="24">
@@ -957,13 +1000,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D24" t="n">
-        <v>46.33</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="E24" t="n">
         <v>-10.93</v>
@@ -976,13 +1019,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>-40.3</v>
+        <v>-85.01000000000001</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -1021,13 +1064,13 @@
         </is>
       </c>
       <c r="B28" t="n">
+        <v>11</v>
+      </c>
+      <c r="C28" t="n">
         <v>7</v>
       </c>
-      <c r="C28" t="n">
-        <v>5</v>
-      </c>
       <c r="D28" t="n">
-        <v>110.32</v>
+        <v>90.47</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1040,16 +1083,16 @@
         </is>
       </c>
       <c r="B29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" t="n">
         <v>4</v>
       </c>
-      <c r="C29" t="n">
-        <v>3</v>
-      </c>
       <c r="D29" t="n">
-        <v>69.44</v>
+        <v>112.56</v>
       </c>
       <c r="E29" t="n">
-        <v>28.44</v>
+        <v>39.94</v>
       </c>
     </row>
     <row r="31">
@@ -1120,13 +1163,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>11.08</v>
+        <v>22.58</v>
       </c>
     </row>
     <row r="38">
@@ -1158,13 +1201,13 @@
         </is>
       </c>
       <c r="B39" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" t="n">
         <v>4</v>
       </c>
-      <c r="C39" t="n">
-        <v>3</v>
-      </c>
       <c r="D39" t="n">
-        <v>28.44</v>
+        <v>39.94</v>
       </c>
     </row>
     <row r="41">
@@ -1237,150 +1280,182 @@
         <v>39.37</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>11.5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" t="n">
-        <v>39.37</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C48" t="n">
         <v>2</v>
       </c>
       <c r="D48" t="n">
+        <v>50.87</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>3</v>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" t="n">
         <v>-10.93</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>3</v>
-      </c>
-      <c r="C51" t="n">
-        <v>3</v>
-      </c>
-      <c r="D51" t="n">
-        <v>58.44</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="n">
+        <v>58.44</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>0.15–0.20%</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="B53" t="n">
         <v>1</v>
       </c>
-      <c r="C52" t="n">
+      <c r="C53" t="n">
         <v>0</v>
       </c>
-      <c r="D52" t="n">
+      <c r="D53" t="n">
         <v>-30</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B57" t="n">
+        <v>5</v>
+      </c>
+      <c r="C57" t="n">
         <v>4</v>
       </c>
-      <c r="C55" t="n">
-        <v>3</v>
-      </c>
-      <c r="D55" t="n">
-        <v>28.44</v>
+      <c r="D57" t="n">
+        <v>39.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>